<commit_message>
Filter Step 10 to chapters with population >= 100
Minimal exclusion: only 2 SJSP chapters (combined pop = 40)
- More inclusive than P_k threshold approach
- Retains all substantive chapters including small ones
- 109 chapters analyzed (was 111)

Updated results:
- Correlations: ρ = -0.46 for demand per capita ↔ SPAR (p < 0.001)
- 4 zero-access chapters: Navajo Mountain (#8), Black Mesa (#12), Alamo (#14), LeChee (#17)
- Pueblo Pintado now included in priority rankings (#19)

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs_tables/10_intervention_priorities.xlsx
+++ b/outputs_tables/10_intervention_priorities.xlsx
@@ -353,7 +353,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I112"/>
+  <dimension ref="A1:I110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -418,7 +418,7 @@
         </is>
       </c>
       <c r="D2">
-        <v>75.70863412861235</v>
+        <v>74.94182621020946</v>
       </c>
       <c r="E2">
         <v>0.02790761417339117</v>
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="D3">
-        <v>72.40809335008936</v>
+        <v>71.59945099767819</v>
       </c>
       <c r="E3">
         <v>0.0255251569552443</v>
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="D4">
-        <v>71.58195372620985</v>
+        <v>70.98298385770426</v>
       </c>
       <c r="E4">
         <v>0.02641513027901684</v>
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="D5">
-        <v>70.4928045706348</v>
+        <v>69.65884842347617</v>
       </c>
       <c r="E5">
         <v>0.03780029128003148</v>
@@ -541,7 +541,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>San Juan Southern Paiute Northern Area</t>
+          <t>Forest Lake Chapter</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -550,22 +550,22 @@
         </is>
       </c>
       <c r="D6">
-        <v>69.23596108706114</v>
+        <v>67.55312773929485</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>0.1100470167361039</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>3.912259564620629E-06</v>
       </c>
       <c r="G6">
-        <v>830.334731754524</v>
+        <v>15069.52640855043</v>
       </c>
       <c r="H6">
-        <v>30.75313821313052</v>
+        <v>28.97985847798159</v>
       </c>
       <c r="I6">
-        <v>27</v>
+        <v>520</v>
       </c>
     </row>
     <row r="7">
@@ -574,7 +574,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Forest Lake Chapter</t>
+          <t>Red Valley Chapter</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -583,22 +583,22 @@
         </is>
       </c>
       <c r="D7">
-        <v>68.44069970135709</v>
+        <v>67.15257387412949</v>
       </c>
       <c r="E7">
-        <v>0.1100470167361039</v>
+        <v>0.2729687088531489</v>
       </c>
       <c r="F7">
-        <v>3.912259564620629E-06</v>
+        <v>9.704256178191467E-06</v>
       </c>
       <c r="G7">
-        <v>15069.52640855043</v>
+        <v>32185.96187861314</v>
       </c>
       <c r="H7">
-        <v>28.97985847798159</v>
+        <v>27.81846316215483</v>
       </c>
       <c r="I7">
-        <v>520</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="8">
@@ -607,7 +607,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Red Valley Chapter</t>
+          <t>Sanostee Chapter</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -616,22 +616,22 @@
         </is>
       </c>
       <c r="D8">
-        <v>67.92898511521378</v>
+        <v>65.35382228266836</v>
       </c>
       <c r="E8">
-        <v>0.2729687088531489</v>
+        <v>0.3111560678000171</v>
       </c>
       <c r="F8">
-        <v>9.704256178191467E-06</v>
+        <v>1.1061847367108E-05</v>
       </c>
       <c r="G8">
-        <v>32185.96187861314</v>
+        <v>38486.47768994235</v>
       </c>
       <c r="H8">
-        <v>27.81846316215483</v>
+        <v>25.35341086293963</v>
       </c>
       <c r="I8">
-        <v>1157</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="9">
@@ -640,7 +640,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Sanostee Chapter</t>
+          <t>Navajo Mountain Chapter</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -649,22 +649,22 @@
         </is>
       </c>
       <c r="D9">
-        <v>66.08931554866695</v>
+        <v>65.13799451820697</v>
       </c>
       <c r="E9">
-        <v>0.3111560678000171</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>1.1061847367108E-05</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>38486.47768994235</v>
+        <v>16543.10150075928</v>
       </c>
       <c r="H9">
-        <v>25.35341086293963</v>
+        <v>24.36391973602251</v>
       </c>
       <c r="I9">
-        <v>1518</v>
+        <v>679</v>
       </c>
     </row>
     <row r="10">
@@ -673,7 +673,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Navajo Mountain Chapter</t>
+          <t>Two Grey Hills Chapter</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -682,22 +682,22 @@
         </is>
       </c>
       <c r="D10">
-        <v>66.01599651636218</v>
+        <v>65.12219550120108</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>0.2164662194647601</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>7.695547436320794E-06</v>
       </c>
       <c r="G10">
-        <v>16543.10150075928</v>
+        <v>28110.28515343216</v>
       </c>
       <c r="H10">
-        <v>24.36391973602251</v>
+        <v>25.6480703954673</v>
       </c>
       <c r="I10">
-        <v>679</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="11">
@@ -706,7 +706,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Two Grey Hills Chapter</t>
+          <t>White Cone Chapter</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -715,22 +715,22 @@
         </is>
       </c>
       <c r="D11">
-        <v>65.92507575588557</v>
+        <v>64.54801279647572</v>
       </c>
       <c r="E11">
-        <v>0.2164662194647601</v>
+        <v>0.362665568774936</v>
       </c>
       <c r="F11">
-        <v>7.695547436320794E-06</v>
+        <v>1.289305137276688E-05</v>
       </c>
       <c r="G11">
-        <v>28110.28515343216</v>
+        <v>32321.42679388845</v>
       </c>
       <c r="H11">
-        <v>25.6480703954673</v>
+        <v>26.68986523029599</v>
       </c>
       <c r="I11">
-        <v>1096</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="12">
@@ -739,7 +739,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>White Cone Chapter</t>
+          <t>Rock Point Chapter</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -748,22 +748,22 @@
         </is>
       </c>
       <c r="D12">
-        <v>65.32354427625249</v>
+        <v>63.59096431927537</v>
       </c>
       <c r="E12">
-        <v>0.362665568774936</v>
+        <v>0.1236891710205495</v>
       </c>
       <c r="F12">
-        <v>1.289305137276688E-05</v>
+        <v>4.397249073326162E-06</v>
       </c>
       <c r="G12">
-        <v>32321.42679388845</v>
+        <v>29102.2946839086</v>
       </c>
       <c r="H12">
-        <v>26.68986523029599</v>
+        <v>22.31771064716918</v>
       </c>
       <c r="I12">
-        <v>1211</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="13">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D13">
-        <v>64.50594027921095</v>
+        <v>63.59003478683287</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="D14">
-        <v>64.40424845570614</v>
+        <v>63.54659869636037</v>
       </c>
       <c r="E14">
         <v>0.2060524923399882</v>
@@ -838,7 +838,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Rock Point Chapter</t>
+          <t>Alamo Chapter</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -847,22 +847,22 @@
         </is>
       </c>
       <c r="D15">
-        <v>64.3874020821912</v>
+        <v>63.32130222293411</v>
       </c>
       <c r="E15">
-        <v>0.1236891710205495</v>
+        <v>0</v>
       </c>
       <c r="F15">
-        <v>4.397249073326162E-06</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>29102.2946839086</v>
+        <v>30124.31763277619</v>
       </c>
       <c r="H15">
-        <v>22.31771064716918</v>
+        <v>19.72777841046247</v>
       </c>
       <c r="I15">
-        <v>1304</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="16">
@@ -871,7 +871,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alamo Chapter</t>
+          <t>Crystal Chapter</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -880,22 +880,22 @@
         </is>
       </c>
       <c r="D16">
-        <v>64.11110257538847</v>
+        <v>63.11526685265701</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>0.3047001171727763</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>1.083233315273626E-05</v>
       </c>
       <c r="G16">
-        <v>30124.31763277619</v>
+        <v>17290.56811975461</v>
       </c>
       <c r="H16">
-        <v>19.72777841046247</v>
+        <v>27.35849386037122</v>
       </c>
       <c r="I16">
-        <v>1527</v>
+        <v>632</v>
       </c>
     </row>
     <row r="17">
@@ -904,7 +904,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Crystal Chapter</t>
+          <t>Sheep Springs Chapter</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -913,22 +913,22 @@
         </is>
       </c>
       <c r="D17">
-        <v>63.98841451484843</v>
+        <v>62.95957495615141</v>
       </c>
       <c r="E17">
-        <v>0.3047001171727763</v>
+        <v>0.2284935461638709</v>
       </c>
       <c r="F17">
-        <v>1.083233315273626E-05</v>
+        <v>8.12312853130177E-06</v>
       </c>
       <c r="G17">
-        <v>17290.56811975461</v>
+        <v>17096.64472023444</v>
       </c>
       <c r="H17">
-        <v>27.35849386037122</v>
+        <v>25.94331520521159</v>
       </c>
       <c r="I17">
-        <v>632</v>
+        <v>659</v>
       </c>
     </row>
     <row r="18">
@@ -937,7 +937,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Sheep Springs Chapter</t>
+          <t>LeChee Chapter</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -946,22 +946,22 @@
         </is>
       </c>
       <c r="D18">
-        <v>63.83398203155086</v>
+        <v>62.85486561350199</v>
       </c>
       <c r="E18">
-        <v>0.2284935461638709</v>
+        <v>0</v>
       </c>
       <c r="F18">
-        <v>8.12312853130177E-06</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>17096.64472023444</v>
+        <v>29178.39472610469</v>
       </c>
       <c r="H18">
-        <v>25.94331520521159</v>
+        <v>19.45226315073646</v>
       </c>
       <c r="I18">
-        <v>659</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="19">
@@ -970,7 +970,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>LeChee Chapter</t>
+          <t>Tolani Lake Chapter</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -979,22 +979,22 @@
         </is>
       </c>
       <c r="D19">
-        <v>63.6508091534488</v>
+        <v>62.73576286494306</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>0.175835372788674</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>6.251088302018776E-06</v>
       </c>
       <c r="G19">
-        <v>29178.39472610469</v>
+        <v>14321.73217930125</v>
       </c>
       <c r="H19">
-        <v>19.45226315073646</v>
+        <v>25.39314216188165</v>
       </c>
       <c r="I19">
-        <v>1500</v>
+        <v>564</v>
       </c>
     </row>
     <row r="20">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Tolani Lake Chapter</t>
+          <t>Pueblo Pintado Chapter</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1012,22 +1012,22 @@
         </is>
       </c>
       <c r="D20">
-        <v>63.6281912905962</v>
+        <v>62.47887157974286</v>
       </c>
       <c r="E20">
-        <v>0.175835372788674</v>
+        <v>0.02788474455638316</v>
       </c>
       <c r="F20">
-        <v>6.251088302018776E-06</v>
+        <v>9.913249975628126E-07</v>
       </c>
       <c r="G20">
-        <v>14321.73217930125</v>
+        <v>7922.286770869622</v>
       </c>
       <c r="H20">
-        <v>25.39314216188165</v>
+        <v>23.93440112045203</v>
       </c>
       <c r="I20">
-        <v>564</v>
+        <v>331</v>
       </c>
     </row>
     <row r="21">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pueblo Pintado Chapter</t>
+          <t>Teec Nos Pos Chapter</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1045,22 +1045,22 @@
         </is>
       </c>
       <c r="D21">
-        <v>63.41286046736861</v>
+        <v>61.92107358643705</v>
       </c>
       <c r="E21">
-        <v>0.02788474455638316</v>
+        <v>0.5399597306803309</v>
       </c>
       <c r="F21">
-        <v>9.913249975628126E-07</v>
+        <v>1.919600079600388E-05</v>
       </c>
       <c r="G21">
-        <v>7922.286770869622</v>
+        <v>27189.85420344533</v>
       </c>
       <c r="H21">
-        <v>23.93440112045203</v>
+        <v>28.11773961059497</v>
       </c>
       <c r="I21">
-        <v>331</v>
+        <v>967</v>
       </c>
     </row>
     <row r="22">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Teec Nos Pos Chapter</t>
+          <t>Newcomb Chapter</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1078,22 +1078,22 @@
         </is>
       </c>
       <c r="D22">
-        <v>62.72993147403406</v>
+        <v>61.55686326334232</v>
       </c>
       <c r="E22">
-        <v>0.5399597306803309</v>
+        <v>0.2348422721175939</v>
       </c>
       <c r="F22">
-        <v>1.919600079600388E-05</v>
+        <v>8.348830822670287E-06</v>
       </c>
       <c r="G22">
-        <v>27189.85420344533</v>
+        <v>13729.27789953941</v>
       </c>
       <c r="H22">
-        <v>28.11773961059497</v>
+        <v>25.33077103236054</v>
       </c>
       <c r="I22">
-        <v>967</v>
+        <v>542</v>
       </c>
     </row>
     <row r="23">
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="D23">
-        <v>62.4730911512703</v>
+        <v>61.52135793375467</v>
       </c>
       <c r="E23">
         <v>0.5042704924866437</v>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Newcomb Chapter</t>
+          <t>Coppermine Chapter</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1144,22 +1144,22 @@
         </is>
       </c>
       <c r="D24">
-        <v>62.45313931515571</v>
+        <v>61.44828959676161</v>
       </c>
       <c r="E24">
-        <v>0.2348422721175939</v>
+        <v>0.2446657766426663</v>
       </c>
       <c r="F24">
-        <v>8.348830822670287E-06</v>
+        <v>8.698064274663536E-06</v>
       </c>
       <c r="G24">
-        <v>13729.27789953941</v>
+        <v>13917.03075059227</v>
       </c>
       <c r="H24">
-        <v>25.33077103236054</v>
+        <v>25.34978278796407</v>
       </c>
       <c r="I24">
-        <v>542</v>
+        <v>549</v>
       </c>
     </row>
     <row r="25">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Coppermine Chapter</t>
+          <t>Naschitti Chapter</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1177,22 +1177,22 @@
         </is>
       </c>
       <c r="D25">
-        <v>62.34334630928412</v>
+        <v>61.31091998175722</v>
       </c>
       <c r="E25">
-        <v>0.2446657766426663</v>
+        <v>0.5891119262702047</v>
       </c>
       <c r="F25">
-        <v>8.698064274663536E-06</v>
+        <v>2.094340070762276E-05</v>
       </c>
       <c r="G25">
-        <v>13917.03075059227</v>
+        <v>35094.29051480199</v>
       </c>
       <c r="H25">
-        <v>25.34978278796407</v>
+        <v>26.70798364901217</v>
       </c>
       <c r="I25">
-        <v>549</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="26">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Naschitti Chapter</t>
+          <t>Tachee Chapter</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1210,22 +1210,22 @@
         </is>
       </c>
       <c r="D26">
-        <v>62.0684434171062</v>
+        <v>60.67337132071897</v>
       </c>
       <c r="E26">
-        <v>0.5891119262702047</v>
+        <v>0.4414192455983922</v>
       </c>
       <c r="F26">
-        <v>2.094340070762276E-05</v>
+        <v>1.569280764549214E-05</v>
       </c>
       <c r="G26">
-        <v>35094.29051480199</v>
+        <v>27685.79827066313</v>
       </c>
       <c r="H26">
-        <v>26.70798364901217</v>
+        <v>25.07771582487603</v>
       </c>
       <c r="I26">
-        <v>1314</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="27">
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="D27">
-        <v>61.51057980000954</v>
+        <v>60.65248576245658</v>
       </c>
       <c r="E27">
         <v>0.4345099181530095</v>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tachee Chapter</t>
+          <t>Sweetwater Chapter</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1276,22 +1276,22 @@
         </is>
       </c>
       <c r="D28">
-        <v>61.47900835662797</v>
+        <v>60.63182316696785</v>
       </c>
       <c r="E28">
-        <v>0.4414192455983922</v>
+        <v>0.2402430718973105</v>
       </c>
       <c r="F28">
-        <v>1.569280764549214E-05</v>
+        <v>8.540833579505268E-06</v>
       </c>
       <c r="G28">
-        <v>27685.79827066313</v>
+        <v>25376.37464446393</v>
       </c>
       <c r="H28">
-        <v>25.07771582487603</v>
+        <v>22.08561761920273</v>
       </c>
       <c r="I28">
-        <v>1104</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="29">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sweetwater Chapter</t>
+          <t>Hard Rock Chapter</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1309,22 +1309,22 @@
         </is>
       </c>
       <c r="D29">
-        <v>61.45245848892657</v>
+        <v>60.30416944566461</v>
       </c>
       <c r="E29">
-        <v>0.2402430718973105</v>
+        <v>0.5016967677893962</v>
       </c>
       <c r="F29">
-        <v>8.540833579505268E-06</v>
+        <v>1.783572182633625E-05</v>
       </c>
       <c r="G29">
-        <v>25376.37464446393</v>
+        <v>25349.03610989268</v>
       </c>
       <c r="H29">
-        <v>22.08561761920273</v>
+        <v>26.2141014580069</v>
       </c>
       <c r="I29">
-        <v>1149</v>
+        <v>967</v>
       </c>
     </row>
     <row r="30">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Hard Rock Chapter</t>
+          <t>White Rock Chapter</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1342,22 +1342,22 @@
         </is>
       </c>
       <c r="D30">
-        <v>61.12498231459091</v>
+        <v>59.34290803451282</v>
       </c>
       <c r="E30">
-        <v>0.5016967677893962</v>
+        <v>0.4742943961862794</v>
       </c>
       <c r="F30">
-        <v>1.783572182633625E-05</v>
+        <v>1.686154557352003E-05</v>
       </c>
       <c r="G30">
-        <v>25349.03610989268</v>
+        <v>5957.275037879956</v>
       </c>
       <c r="H30">
-        <v>26.2141014580069</v>
+        <v>28.77910646318819</v>
       </c>
       <c r="I30">
-        <v>967</v>
+        <v>207</v>
       </c>
     </row>
     <row r="31">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>White Rock Chapter</t>
+          <t>Cove Chapter</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D31">
-        <v>60.28965846477118</v>
+        <v>59.30501797749366</v>
       </c>
       <c r="E31">
-        <v>0.4742943961862794</v>
+        <v>0.1055426132151874</v>
       </c>
       <c r="F31">
-        <v>1.686154557352003E-05</v>
+        <v>3.75212441257125E-06</v>
       </c>
       <c r="G31">
-        <v>5957.275037879956</v>
+        <v>7999.851318430388</v>
       </c>
       <c r="H31">
-        <v>28.77910646318819</v>
+        <v>22.03815790201209</v>
       </c>
       <c r="I31">
-        <v>207</v>
+        <v>363</v>
       </c>
     </row>
     <row r="32">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Cove Chapter</t>
+          <t>Burnham Chapter</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1408,22 +1408,22 @@
         </is>
       </c>
       <c r="D32">
-        <v>60.23850313108879</v>
+        <v>59.21607569049385</v>
       </c>
       <c r="E32">
-        <v>0.1055426132151874</v>
+        <v>0.2575990231478117</v>
       </c>
       <c r="F32">
-        <v>3.75212441257125E-06</v>
+        <v>9.157851544160242E-06</v>
       </c>
       <c r="G32">
-        <v>7999.851318430388</v>
+        <v>5030.260911247553</v>
       </c>
       <c r="H32">
-        <v>22.03815790201209</v>
+        <v>25.15130455623776</v>
       </c>
       <c r="I32">
-        <v>363</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Burnham Chapter</t>
+          <t>Kaibeto Chapter</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1441,22 +1441,22 @@
         </is>
       </c>
       <c r="D33">
-        <v>60.16884650734808</v>
+        <v>58.69550529309917</v>
       </c>
       <c r="E33">
-        <v>0.2575990231478117</v>
+        <v>0.09478939147055138</v>
       </c>
       <c r="F33">
-        <v>9.157851544160242E-06</v>
+        <v>3.369838768955644E-06</v>
       </c>
       <c r="G33">
-        <v>5030.260911247553</v>
+        <v>31313.14846006263</v>
       </c>
       <c r="H33">
-        <v>25.15130455623776</v>
+        <v>16.42872427075689</v>
       </c>
       <c r="I33">
-        <v>200</v>
+        <v>1906</v>
       </c>
     </row>
     <row r="34">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Kaibeto Chapter</t>
+          <t>Shiprock Chapter</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1474,22 +1474,22 @@
         </is>
       </c>
       <c r="D34">
-        <v>59.47758492051629</v>
+        <v>58.55488837829027</v>
       </c>
       <c r="E34">
-        <v>0.09478939147055138</v>
+        <v>1.688894285085774</v>
       </c>
       <c r="F34">
-        <v>3.369838768955644E-06</v>
+        <v>6.004154420927797E-05</v>
       </c>
       <c r="G34">
-        <v>31313.14846006263</v>
+        <v>151737.1197816597</v>
       </c>
       <c r="H34">
-        <v>16.42872427075689</v>
+        <v>18.58840129629544</v>
       </c>
       <c r="I34">
-        <v>1906</v>
+        <v>8163</v>
       </c>
     </row>
     <row r="35">
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="D35">
-        <v>59.1225960628278</v>
+        <v>58.20106071302942</v>
       </c>
       <c r="E35">
         <v>0.2683325572254379</v>
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="D36">
-        <v>58.90372648825749</v>
+        <v>58.0424759750465</v>
       </c>
       <c r="E36">
         <v>0.5870303690139005</v>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="D37">
-        <v>58.83266384210392</v>
+        <v>57.97255096755315</v>
       </c>
       <c r="E37">
         <v>0.4108525097421717</v>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="D38">
-        <v>58.66372471609631</v>
+        <v>57.88739419153136</v>
       </c>
       <c r="E38">
         <v>0.4108077222772788</v>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Shiprock Chapter</t>
+          <t>Houck Chapter</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1639,22 +1639,22 @@
         </is>
       </c>
       <c r="D39">
-        <v>58.55488837829027</v>
+        <v>56.01474769186691</v>
       </c>
       <c r="E39">
-        <v>1.688894285085774</v>
+        <v>0.7954068047890792</v>
       </c>
       <c r="F39">
-        <v>6.004154420927797E-05</v>
+        <v>2.827734882866194E-05</v>
       </c>
       <c r="G39">
-        <v>151737.1197816597</v>
+        <v>32962.69462770235</v>
       </c>
       <c r="H39">
-        <v>18.58840129629544</v>
+        <v>25.31696976014005</v>
       </c>
       <c r="I39">
-        <v>8163</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="40">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Houck Chapter</t>
+          <t>Counselor Chapter</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1672,22 +1672,22 @@
         </is>
       </c>
       <c r="D40">
-        <v>56.78611453147246</v>
+        <v>54.92269120574767</v>
       </c>
       <c r="E40">
-        <v>0.7954068047890792</v>
+        <v>0.6537820678534564</v>
       </c>
       <c r="F40">
-        <v>2.827734882866194E-05</v>
+        <v>2.324247602523143E-05</v>
       </c>
       <c r="G40">
-        <v>32962.69462770235</v>
+        <v>19197.11711816966</v>
       </c>
       <c r="H40">
-        <v>25.31696976014005</v>
+        <v>24.64328256504449</v>
       </c>
       <c r="I40">
-        <v>1302</v>
+        <v>779</v>
       </c>
     </row>
     <row r="41">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Counselor Chapter</t>
+          <t>St. Michaels Chapter</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1705,22 +1705,22 @@
         </is>
       </c>
       <c r="D41">
-        <v>55.78345700481027</v>
+        <v>54.80041390910053</v>
       </c>
       <c r="E41">
-        <v>0.6537820678534564</v>
+        <v>1.449495087236773</v>
       </c>
       <c r="F41">
-        <v>2.324247602523143E-05</v>
+        <v>5.153071102791844E-05</v>
       </c>
       <c r="G41">
-        <v>19197.11711816966</v>
+        <v>105339.4768735656</v>
       </c>
       <c r="H41">
-        <v>24.64328256504449</v>
+        <v>20.29662367506082</v>
       </c>
       <c r="I41">
-        <v>779</v>
+        <v>5190</v>
       </c>
     </row>
     <row r="42">
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="D42">
-        <v>55.54814854761351</v>
+        <v>54.72748899843938</v>
       </c>
       <c r="E42">
         <v>0.613956923048127</v>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>St. Michaels Chapter</t>
+          <t>Dilcon Chapter</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1771,22 +1771,22 @@
         </is>
       </c>
       <c r="D43">
-        <v>55.10173806309052</v>
+        <v>53.94298877981377</v>
       </c>
       <c r="E43">
-        <v>1.449495087236773</v>
+        <v>0.9663861463119082</v>
       </c>
       <c r="F43">
-        <v>5.153071102791844E-05</v>
+        <v>3.435580133073481E-05</v>
       </c>
       <c r="G43">
-        <v>105339.4768735656</v>
+        <v>47339.60151338952</v>
       </c>
       <c r="H43">
-        <v>20.29662367506082</v>
+        <v>23.17161111766496</v>
       </c>
       <c r="I43">
-        <v>5190</v>
+        <v>2043</v>
       </c>
     </row>
     <row r="44">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dilcon Chapter</t>
+          <t>Ramah Chapter</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1804,22 +1804,22 @@
         </is>
       </c>
       <c r="D44">
-        <v>54.62098645166002</v>
+        <v>53.78844442194043</v>
       </c>
       <c r="E44">
-        <v>0.9663861463119082</v>
+        <v>0.7403564994274383</v>
       </c>
       <c r="F44">
-        <v>3.435580133073481E-05</v>
+        <v>2.632026639177198E-05</v>
       </c>
       <c r="G44">
-        <v>47339.60151338952</v>
+        <v>44849.42944764543</v>
       </c>
       <c r="H44">
-        <v>23.17161111766496</v>
+        <v>19.67943371989707</v>
       </c>
       <c r="I44">
-        <v>2043</v>
+        <v>2279</v>
       </c>
     </row>
     <row r="45">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ramah Chapter</t>
+          <t>Fort Defiance Chapter</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1837,22 +1837,22 @@
         </is>
       </c>
       <c r="D45">
-        <v>54.48261422978258</v>
+        <v>53.56873927644879</v>
       </c>
       <c r="E45">
-        <v>0.7403564994274383</v>
+        <v>1.404761229638005</v>
       </c>
       <c r="F45">
-        <v>2.632026639177198E-05</v>
+        <v>4.994038656984761E-05</v>
       </c>
       <c r="G45">
-        <v>44849.42944764543</v>
+        <v>101676.2320595608</v>
       </c>
       <c r="H45">
-        <v>19.67943371989707</v>
+        <v>19.04762683768469</v>
       </c>
       <c r="I45">
-        <v>2279</v>
+        <v>5338</v>
       </c>
     </row>
     <row r="46">
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="D46">
-        <v>54.01346239846567</v>
+        <v>53.22135347965484</v>
       </c>
       <c r="E46">
         <v>0.8590881279066566</v>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="D47">
-        <v>53.97183986211921</v>
+        <v>53.19699213518186</v>
       </c>
       <c r="E47">
         <v>0.7860835528434029</v>
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="D48">
-        <v>53.96093083106781</v>
+        <v>53.07386805863713</v>
       </c>
       <c r="E48">
         <v>0.2979892134591955</v>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Fort Defiance Chapter</t>
+          <t>Huerfano Chapter</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1969,22 +1969,22 @@
         </is>
       </c>
       <c r="D49">
-        <v>53.89385395244062</v>
+        <v>53.00054693136042</v>
       </c>
       <c r="E49">
-        <v>1.404761229638005</v>
+        <v>0.8339999051546039</v>
       </c>
       <c r="F49">
-        <v>4.994038656984761E-05</v>
+        <v>2.964936444990731E-05</v>
       </c>
       <c r="G49">
-        <v>101676.2320595608</v>
+        <v>47432.38914495373</v>
       </c>
       <c r="H49">
-        <v>19.04762683768469</v>
+        <v>19.94633689863487</v>
       </c>
       <c r="I49">
-        <v>5338</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="50">
@@ -1993,7 +1993,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Huerfano Chapter</t>
+          <t>Lukachukai Chapter</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2002,22 +2002,22 @@
         </is>
       </c>
       <c r="D50">
-        <v>53.67794200460833</v>
+        <v>52.63647876051242</v>
       </c>
       <c r="E50">
-        <v>0.8339999051546039</v>
+        <v>0.7020893273181287</v>
       </c>
       <c r="F50">
-        <v>2.964936444990731E-05</v>
+        <v>2.495983778102059E-05</v>
       </c>
       <c r="G50">
-        <v>47432.38914495373</v>
+        <v>35218.47957333992</v>
       </c>
       <c r="H50">
-        <v>19.94633689863487</v>
+        <v>19.85258149568203</v>
       </c>
       <c r="I50">
-        <v>2378</v>
+        <v>1774</v>
       </c>
     </row>
     <row r="51">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Lukachukai Chapter</t>
+          <t>Steamboat Chapter</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2035,22 +2035,22 @@
         </is>
       </c>
       <c r="D51">
-        <v>53.39319566430821</v>
+        <v>52.55333323054739</v>
       </c>
       <c r="E51">
-        <v>0.7020893273181287</v>
+        <v>1.110552125008533</v>
       </c>
       <c r="F51">
-        <v>2.495983778102059E-05</v>
+        <v>3.948101731365678E-05</v>
       </c>
       <c r="G51">
-        <v>35218.47957333992</v>
+        <v>32147.93627407949</v>
       </c>
       <c r="H51">
-        <v>19.85258149568203</v>
+        <v>27.35994576517404</v>
       </c>
       <c r="I51">
-        <v>1774</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="52">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Steamboat Chapter</t>
+          <t>Mariano Lake Chapter</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2068,22 +2068,22 @@
         </is>
       </c>
       <c r="D52">
-        <v>53.32999142454563</v>
+        <v>51.68223087336107</v>
       </c>
       <c r="E52">
-        <v>1.110552125008533</v>
+        <v>0.6681474045819183</v>
       </c>
       <c r="F52">
-        <v>3.948101731365678E-05</v>
+        <v>2.375317524890682E-05</v>
       </c>
       <c r="G52">
-        <v>32147.93627407949</v>
+        <v>18405.09258888919</v>
       </c>
       <c r="H52">
-        <v>27.35994576517404</v>
+        <v>21.78117466140732</v>
       </c>
       <c r="I52">
-        <v>1175</v>
+        <v>845</v>
       </c>
     </row>
     <row r="53">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Mariano Lake Chapter</t>
+          <t>Beclabito Chapter</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2101,22 +2101,22 @@
         </is>
       </c>
       <c r="D53">
-        <v>52.5481403846096</v>
+        <v>51.51122741962475</v>
       </c>
       <c r="E53">
-        <v>0.6681474045819183</v>
+        <v>0.9224382288064679</v>
       </c>
       <c r="F53">
-        <v>2.375317524890682E-05</v>
+        <v>3.279341767231973E-05</v>
       </c>
       <c r="G53">
-        <v>18405.09258888919</v>
+        <v>16812.06380643935</v>
       </c>
       <c r="H53">
-        <v>21.78117466140732</v>
+        <v>26.26884969756148</v>
       </c>
       <c r="I53">
-        <v>845</v>
+        <v>640</v>
       </c>
     </row>
     <row r="54">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Beclabito Chapter</t>
+          <t>Kinlichee Chapter</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2134,22 +2134,22 @@
         </is>
       </c>
       <c r="D54">
-        <v>52.38748267302885</v>
+        <v>51.48820073679918</v>
       </c>
       <c r="E54">
-        <v>0.9224382288064679</v>
+        <v>0.8957372337245202</v>
       </c>
       <c r="F54">
-        <v>3.279341767231973E-05</v>
+        <v>3.184417591645514E-05</v>
       </c>
       <c r="G54">
-        <v>16812.06380643935</v>
+        <v>34596.62847962941</v>
       </c>
       <c r="H54">
-        <v>26.26884969756148</v>
+        <v>22.12060644477583</v>
       </c>
       <c r="I54">
-        <v>640</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="55">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Kinlichee Chapter</t>
+          <t>Oljato Chapter</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2167,22 +2167,22 @@
         </is>
       </c>
       <c r="D55">
-        <v>52.24895618098142</v>
+        <v>50.81908658514779</v>
       </c>
       <c r="E55">
-        <v>0.8957372337245202</v>
+        <v>1.005075341600984</v>
       </c>
       <c r="F55">
-        <v>3.184417591645514E-05</v>
+        <v>3.573123320346001E-05</v>
       </c>
       <c r="G55">
-        <v>34596.62847962941</v>
+        <v>48692.13836335862</v>
       </c>
       <c r="H55">
-        <v>22.12060644477583</v>
+        <v>20.3988849448507</v>
       </c>
       <c r="I55">
-        <v>1564</v>
+        <v>2387</v>
       </c>
     </row>
     <row r="56">
@@ -2200,7 +2200,7 @@
         </is>
       </c>
       <c r="D56">
-        <v>51.60918471370972</v>
+        <v>50.81409440243009</v>
       </c>
       <c r="E56">
         <v>0.9429649471587411</v>
@@ -2224,31 +2224,31 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Oljato Chapter</t>
+          <t>Pinedale Chapter</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Tier 2: High Priority</t>
+          <t>Tier 3: Moderate Priority</t>
         </is>
       </c>
       <c r="D57">
-        <v>51.48830036202624</v>
+        <v>50.51565200759032</v>
       </c>
       <c r="E57">
-        <v>1.005075341600984</v>
+        <v>0.7093279871306061</v>
       </c>
       <c r="F57">
-        <v>3.573123320346001E-05</v>
+        <v>2.521717793367836E-05</v>
       </c>
       <c r="G57">
-        <v>48692.13836335862</v>
+        <v>27583.33922164658</v>
       </c>
       <c r="H57">
-        <v>20.3988849448507</v>
+        <v>19.41121690474777</v>
       </c>
       <c r="I57">
-        <v>2387</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="58">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Pinedale Chapter</t>
+          <t>Cañoncito Chapter</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2266,22 +2266,22 @@
         </is>
       </c>
       <c r="D58">
-        <v>51.32195445200563</v>
+        <v>50.49923441018396</v>
       </c>
       <c r="E58">
-        <v>0.7093279871306061</v>
+        <v>0.7378274123089852</v>
       </c>
       <c r="F58">
-        <v>2.521717793367836E-05</v>
+        <v>2.623035531955586E-05</v>
       </c>
       <c r="G58">
-        <v>27583.33922164658</v>
+        <v>30860.4948663183</v>
       </c>
       <c r="H58">
-        <v>19.41121690474777</v>
+        <v>19.20379269839346</v>
       </c>
       <c r="I58">
-        <v>1421</v>
+        <v>1607</v>
       </c>
     </row>
     <row r="59">
@@ -2299,7 +2299,7 @@
         </is>
       </c>
       <c r="D59">
-        <v>51.30160342486666</v>
+        <v>50.40393054421145</v>
       </c>
       <c r="E59">
         <v>1.015208125107263</v>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Cañoncito Chapter</t>
+          <t>Teesto Chapter</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2332,22 +2332,22 @@
         </is>
       </c>
       <c r="D60">
-        <v>51.28425374428954</v>
+        <v>50.30300003614659</v>
       </c>
       <c r="E60">
-        <v>0.7378274123089852</v>
+        <v>1.059940308181128</v>
       </c>
       <c r="F60">
-        <v>2.623035531955586E-05</v>
+        <v>3.76817266982586E-05</v>
       </c>
       <c r="G60">
-        <v>30860.4948663183</v>
+        <v>21281.35736212334</v>
       </c>
       <c r="H60">
-        <v>19.20379269839346</v>
+        <v>26.46934995288972</v>
       </c>
       <c r="I60">
-        <v>1607</v>
+        <v>804</v>
       </c>
     </row>
     <row r="61">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Teesto Chapter</t>
+          <t>Inscription House Chapter</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2365,22 +2365,22 @@
         </is>
       </c>
       <c r="D61">
-        <v>51.15022997672894</v>
+        <v>49.82803333015621</v>
       </c>
       <c r="E61">
-        <v>1.059940308181128</v>
+        <v>0.8360036111371272</v>
       </c>
       <c r="F61">
-        <v>3.76817266982586E-05</v>
+        <v>2.972059780204454E-05</v>
       </c>
       <c r="G61">
-        <v>21281.35736212334</v>
+        <v>23552.04972724615</v>
       </c>
       <c r="H61">
-        <v>26.46934995288972</v>
+        <v>21.70695827395959</v>
       </c>
       <c r="I61">
-        <v>804</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="62">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Inscription House Chapter</t>
+          <t>Nahatadziil Chapter</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2398,22 +2398,22 @@
         </is>
       </c>
       <c r="D62">
-        <v>50.660516520408</v>
+        <v>49.28216749582225</v>
       </c>
       <c r="E62">
-        <v>0.8360036111371272</v>
+        <v>0.9559845876303178</v>
       </c>
       <c r="F62">
-        <v>2.972059780204454E-05</v>
+        <v>3.398601759060306E-05</v>
       </c>
       <c r="G62">
-        <v>23552.04972724615</v>
+        <v>35985.5199723685</v>
       </c>
       <c r="H62">
-        <v>21.70695827395959</v>
+        <v>20.63389906672506</v>
       </c>
       <c r="I62">
-        <v>1085</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="63">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Nahatadziil Chapter</t>
+          <t>Whippoorwill Chapter</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2431,22 +2431,22 @@
         </is>
       </c>
       <c r="D63">
-        <v>50.03390294399171</v>
+        <v>49.07058688278449</v>
       </c>
       <c r="E63">
-        <v>0.9559845876303178</v>
+        <v>0.6552443027657574</v>
       </c>
       <c r="F63">
-        <v>3.398601759060306E-05</v>
+        <v>2.329445964724175E-05</v>
       </c>
       <c r="G63">
-        <v>35985.5199723685</v>
+        <v>22393.08276468831</v>
       </c>
       <c r="H63">
-        <v>20.63389906672506</v>
+        <v>18.10273465213283</v>
       </c>
       <c r="I63">
-        <v>1744</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="64">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Whippoorwill Chapter</t>
+          <t>Mexican Water Chapter</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2464,22 +2464,22 @@
         </is>
       </c>
       <c r="D64">
-        <v>49.91059685063977</v>
+        <v>48.98461868276473</v>
       </c>
       <c r="E64">
-        <v>0.6552443027657574</v>
+        <v>0.9661568437445235</v>
       </c>
       <c r="F64">
-        <v>2.329445964724175E-05</v>
+        <v>3.434764944085128E-05</v>
       </c>
       <c r="G64">
-        <v>22393.08276468831</v>
+        <v>18100.03120255824</v>
       </c>
       <c r="H64">
-        <v>18.10273465213283</v>
+        <v>24.19790267721689</v>
       </c>
       <c r="I64">
-        <v>1237</v>
+        <v>748</v>
       </c>
     </row>
     <row r="65">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Mexican Water Chapter</t>
+          <t>Ganado Chapter</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2497,22 +2497,22 @@
         </is>
       </c>
       <c r="D65">
-        <v>49.85250938009061</v>
+        <v>48.66227120672027</v>
       </c>
       <c r="E65">
-        <v>0.9661568437445235</v>
+        <v>1.241736761548638</v>
       </c>
       <c r="F65">
-        <v>3.434764944085128E-05</v>
+        <v>4.414473618816336E-05</v>
       </c>
       <c r="G65">
-        <v>18100.03120255824</v>
+        <v>47481.80036658785</v>
       </c>
       <c r="H65">
-        <v>24.19790267721689</v>
+        <v>22.50322292255348</v>
       </c>
       <c r="I65">
-        <v>748</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="66">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Coyote Canyon Chapter</t>
+          <t>Aneth Chapter</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2530,22 +2530,22 @@
         </is>
       </c>
       <c r="D66">
-        <v>49.38837788010072</v>
+        <v>48.61470794153384</v>
       </c>
       <c r="E66">
-        <v>1.102200034389966</v>
+        <v>1.180747336751176</v>
       </c>
       <c r="F66">
-        <v>3.918409380426784E-05</v>
+        <v>4.19765132996068E-05</v>
       </c>
       <c r="G66">
-        <v>19616.73996910575</v>
+        <v>42860.86338418152</v>
       </c>
       <c r="H66">
-        <v>25.74375324029626</v>
+        <v>22.3699704510342</v>
       </c>
       <c r="I66">
-        <v>762</v>
+        <v>1916</v>
       </c>
     </row>
     <row r="67">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Ganado Chapter</t>
+          <t>Coyote Canyon Chapter</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2563,22 +2563,22 @@
         </is>
       </c>
       <c r="D67">
-        <v>49.33934538447385</v>
+        <v>48.53033727336747</v>
       </c>
       <c r="E67">
-        <v>1.241736761548638</v>
+        <v>1.102200034389966</v>
       </c>
       <c r="F67">
-        <v>4.414473618816336E-05</v>
+        <v>3.918409380426784E-05</v>
       </c>
       <c r="G67">
-        <v>47481.80036658785</v>
+        <v>19616.73996910575</v>
       </c>
       <c r="H67">
-        <v>22.50322292255348</v>
+        <v>25.74375324029626</v>
       </c>
       <c r="I67">
-        <v>2110</v>
+        <v>762</v>
       </c>
     </row>
     <row r="68">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Aneth Chapter</t>
+          <t>Standing Rock Chapter</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2596,22 +2596,22 @@
         </is>
       </c>
       <c r="D68">
-        <v>49.32179226289801</v>
+        <v>48.21592786636047</v>
       </c>
       <c r="E68">
-        <v>1.180747336751176</v>
+        <v>0.9837785432198488</v>
       </c>
       <c r="F68">
-        <v>4.19765132996068E-05</v>
+        <v>3.497411496769543E-05</v>
       </c>
       <c r="G68">
-        <v>42860.86338418152</v>
+        <v>15565.51651662906</v>
       </c>
       <c r="H68">
-        <v>22.3699704510342</v>
+        <v>24.24535282964027</v>
       </c>
       <c r="I68">
-        <v>1916</v>
+        <v>642</v>
       </c>
     </row>
     <row r="69">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Standing Rock Chapter</t>
+          <t>Lupton Chapter</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2629,22 +2629,22 @@
         </is>
       </c>
       <c r="D69">
-        <v>49.10027867772762</v>
+        <v>47.69213879315635</v>
       </c>
       <c r="E69">
-        <v>0.9837785432198488</v>
+        <v>1.093029727277549</v>
       </c>
       <c r="F69">
-        <v>3.497411496769543E-05</v>
+        <v>3.885808204333937E-05</v>
       </c>
       <c r="G69">
-        <v>15565.51651662906</v>
+        <v>18069.01561536165</v>
       </c>
       <c r="H69">
-        <v>24.24535282964027</v>
+        <v>25.06104801021033</v>
       </c>
       <c r="I69">
-        <v>642</v>
+        <v>721</v>
       </c>
     </row>
     <row r="70">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Lupton Chapter</t>
+          <t>Tselani Chapter</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2662,22 +2662,22 @@
         </is>
       </c>
       <c r="D70">
-        <v>48.56023091764504</v>
+        <v>47.53682976561733</v>
       </c>
       <c r="E70">
-        <v>1.093029727277549</v>
+        <v>1.122115570732303</v>
       </c>
       <c r="F70">
-        <v>3.885808204333937E-05</v>
+        <v>3.989210706851379E-05</v>
       </c>
       <c r="G70">
-        <v>18069.01561536165</v>
+        <v>31021.90363853504</v>
       </c>
       <c r="H70">
-        <v>25.06104801021033</v>
+        <v>22.7266693322601</v>
       </c>
       <c r="I70">
-        <v>721</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="71">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Tselani Chapter</t>
+          <t>Tsaile-Wheatfields Chapter</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2695,22 +2695,22 @@
         </is>
       </c>
       <c r="D71">
-        <v>48.32080084902123</v>
+        <v>45.87740788622367</v>
       </c>
       <c r="E71">
-        <v>1.122115570732303</v>
+        <v>0.8440874958353337</v>
       </c>
       <c r="F71">
-        <v>3.989210706851379E-05</v>
+        <v>3.00079863762E-05</v>
       </c>
       <c r="G71">
-        <v>31021.90363853504</v>
+        <v>37849.34626326319</v>
       </c>
       <c r="H71">
-        <v>22.7266693322601</v>
+        <v>14.90718639750421</v>
       </c>
       <c r="I71">
-        <v>1365</v>
+        <v>2539</v>
       </c>
     </row>
     <row r="72">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Tsaile-Wheatfields Chapter</t>
+          <t>Round Rock Chapter</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2728,22 +2728,22 @@
         </is>
       </c>
       <c r="D72">
-        <v>46.61703892897321</v>
+        <v>45.22523363184165</v>
       </c>
       <c r="E72">
-        <v>0.8440874958353337</v>
+        <v>0.8838884273507859</v>
       </c>
       <c r="F72">
-        <v>3.00079863762E-05</v>
+        <v>3.142294136199066E-05</v>
       </c>
       <c r="G72">
-        <v>37849.34626326319</v>
+        <v>19035.3245774455</v>
       </c>
       <c r="H72">
-        <v>14.90718639750421</v>
+        <v>18.80960926625049</v>
       </c>
       <c r="I72">
-        <v>2539</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="73">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Round Rock Chapter</t>
+          <t>Chi Chil Tah Chapter</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2761,22 +2761,22 @@
         </is>
       </c>
       <c r="D73">
-        <v>46.08705017394636</v>
+        <v>43.86367201122776</v>
       </c>
       <c r="E73">
-        <v>0.8838884273507859</v>
+        <v>1.785453640016208</v>
       </c>
       <c r="F73">
-        <v>3.142294136199066E-05</v>
+        <v>6.347430659652273E-05</v>
       </c>
       <c r="G73">
-        <v>19035.3245774455</v>
+        <v>43919.52274514862</v>
       </c>
       <c r="H73">
-        <v>18.80960926625049</v>
+        <v>27.65713019215908</v>
       </c>
       <c r="I73">
-        <v>1012</v>
+        <v>1588</v>
       </c>
     </row>
     <row r="74">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Chi Chil Tah Chapter</t>
+          <t>Bodaway Chapter</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2794,22 +2794,22 @@
         </is>
       </c>
       <c r="D74">
-        <v>44.56388099116697</v>
+        <v>43.72954504576312</v>
       </c>
       <c r="E74">
-        <v>1.785453640016208</v>
+        <v>1.242509678589721</v>
       </c>
       <c r="F74">
-        <v>6.347430659652273E-05</v>
+        <v>4.417221400788369E-05</v>
       </c>
       <c r="G74">
-        <v>43919.52274514862</v>
+        <v>30200.69041664335</v>
       </c>
       <c r="H74">
-        <v>27.65713019215908</v>
+        <v>21.10460546236433</v>
       </c>
       <c r="I74">
-        <v>1588</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="75">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Bodaway Chapter</t>
+          <t>Nageezi Chapter</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2827,22 +2827,22 @@
         </is>
       </c>
       <c r="D75">
-        <v>44.51884940395906</v>
+        <v>43.49447337463818</v>
       </c>
       <c r="E75">
-        <v>1.242509678589721</v>
+        <v>1.244032424965223</v>
       </c>
       <c r="F75">
-        <v>4.417221400788369E-05</v>
+        <v>4.42263488608651E-05</v>
       </c>
       <c r="G75">
-        <v>30200.69041664335</v>
+        <v>21734.79562643881</v>
       </c>
       <c r="H75">
-        <v>21.10460546236433</v>
+        <v>22.64041211087376</v>
       </c>
       <c r="I75">
-        <v>1431</v>
+        <v>960</v>
       </c>
     </row>
     <row r="76">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Nageezi Chapter</t>
+          <t>Red Lake Chapter</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2860,22 +2860,22 @@
         </is>
       </c>
       <c r="D76">
-        <v>44.33875851257933</v>
+        <v>43.12699946223558</v>
       </c>
       <c r="E76">
-        <v>1.244032424965223</v>
+        <v>0.646091957198671</v>
       </c>
       <c r="F76">
-        <v>4.42263488608651E-05</v>
+        <v>2.296908643363241E-05</v>
       </c>
       <c r="G76">
-        <v>21734.79562643881</v>
+        <v>24747.86570329223</v>
       </c>
       <c r="H76">
-        <v>22.64041211087376</v>
+        <v>11.46265201634656</v>
       </c>
       <c r="I76">
-        <v>960</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="77">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Red Lake Chapter</t>
+          <t>Rough Rock Chapter</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2893,22 +2893,22 @@
         </is>
       </c>
       <c r="D77">
-        <v>43.95171656320513</v>
+        <v>42.8920383395095</v>
       </c>
       <c r="E77">
-        <v>0.646091957198671</v>
+        <v>1.074357595621582</v>
       </c>
       <c r="F77">
-        <v>2.296908643363241E-05</v>
+        <v>3.819427281134457E-05</v>
       </c>
       <c r="G77">
-        <v>24747.86570329223</v>
+        <v>15663.50397252518</v>
       </c>
       <c r="H77">
-        <v>11.46265201634656</v>
+        <v>20.39518746422549</v>
       </c>
       <c r="I77">
-        <v>2159</v>
+        <v>768</v>
       </c>
     </row>
     <row r="78">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Rough Rock Chapter</t>
+          <t>Littlewater Chapter</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2926,22 +2926,22 @@
         </is>
       </c>
       <c r="D78">
-        <v>43.77575278261742</v>
+        <v>42.62047871731961</v>
       </c>
       <c r="E78">
-        <v>1.074357595621582</v>
+        <v>1.107843602941287</v>
       </c>
       <c r="F78">
-        <v>3.819427281134457E-05</v>
+        <v>3.938472718532937E-05</v>
       </c>
       <c r="G78">
-        <v>15663.50397252518</v>
+        <v>10823.4854050372</v>
       </c>
       <c r="H78">
-        <v>20.39518746422549</v>
+        <v>21.6903515131006</v>
       </c>
       <c r="I78">
-        <v>768</v>
+        <v>499</v>
       </c>
     </row>
     <row r="79">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Littlewater Chapter</t>
+          <t>Chilchinbeto Chapter</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2959,22 +2959,22 @@
         </is>
       </c>
       <c r="D79">
-        <v>43.53562610418791</v>
+        <v>42.59184343867778</v>
       </c>
       <c r="E79">
-        <v>1.107843602941287</v>
+        <v>1.312836868834997</v>
       </c>
       <c r="F79">
-        <v>3.938472718532937E-05</v>
+        <v>4.667240193528351E-05</v>
       </c>
       <c r="G79">
-        <v>10823.4854050372</v>
+        <v>32177.64887189683</v>
       </c>
       <c r="H79">
-        <v>21.6903515131006</v>
+        <v>20.74638869883741</v>
       </c>
       <c r="I79">
-        <v>499</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="80">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Chilchinbeto Chapter</t>
+          <t>Shonto Chapter</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2992,22 +2992,22 @@
         </is>
       </c>
       <c r="D80">
-        <v>43.36830866762782</v>
+        <v>42.10680365421931</v>
       </c>
       <c r="E80">
-        <v>1.312836868834997</v>
+        <v>1.585026753638292</v>
       </c>
       <c r="F80">
-        <v>4.667240193528351E-05</v>
+        <v>5.634897029486286E-05</v>
       </c>
       <c r="G80">
-        <v>32177.64887189683</v>
+        <v>42251.97525572382</v>
       </c>
       <c r="H80">
-        <v>20.74638869883741</v>
+        <v>22.81424149877096</v>
       </c>
       <c r="I80">
-        <v>1551</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="81">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Shonto Chapter</t>
+          <t>Baca Chapter</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3025,22 +3025,22 @@
         </is>
       </c>
       <c r="D81">
-        <v>42.81784232948343</v>
+        <v>40.53043248368046</v>
       </c>
       <c r="E81">
-        <v>1.585026753638292</v>
+        <v>1.25826602362245</v>
       </c>
       <c r="F81">
-        <v>5.634897029486286E-05</v>
+        <v>4.473236469061938E-05</v>
       </c>
       <c r="G81">
-        <v>42251.97525572382</v>
+        <v>16014.73302472268</v>
       </c>
       <c r="H81">
-        <v>22.81424149877096</v>
+        <v>21.072017137793</v>
       </c>
       <c r="I81">
-        <v>1852</v>
+        <v>760</v>
       </c>
     </row>
     <row r="82">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Baca Chapter</t>
+          <t>Dennehotso Chapter</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3058,22 +3058,22 @@
         </is>
       </c>
       <c r="D82">
-        <v>41.41186591011647</v>
+        <v>40.30165465884575</v>
       </c>
       <c r="E82">
-        <v>1.25826602362245</v>
+        <v>1.514314285861111</v>
       </c>
       <c r="F82">
-        <v>4.473236469061938E-05</v>
+        <v>5.383508544269455E-05</v>
       </c>
       <c r="G82">
-        <v>16014.73302472268</v>
+        <v>31442.71350301213</v>
       </c>
       <c r="H82">
-        <v>21.072017137793</v>
+        <v>22.01870693488245</v>
       </c>
       <c r="I82">
-        <v>760</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="83">
@@ -3091,7 +3091,7 @@
         </is>
       </c>
       <c r="D83">
-        <v>41.16018799017898</v>
+        <v>40.27341515232243</v>
       </c>
       <c r="E83">
         <v>1.451236161749263</v>
@@ -3115,31 +3115,31 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Dennehotso Chapter</t>
+          <t>Church Rock Chapter</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Tier 3: Moderate Priority</t>
+          <t>Tier 4: Lower Priority</t>
         </is>
       </c>
       <c r="D84">
-        <v>41.08289284099742</v>
+        <v>39.86073199443618</v>
       </c>
       <c r="E84">
-        <v>1.514314285861111</v>
+        <v>1.636373562236403</v>
       </c>
       <c r="F84">
-        <v>5.383508544269455E-05</v>
+        <v>5.817439045625099E-05</v>
       </c>
       <c r="G84">
-        <v>31442.71350301213</v>
+        <v>56567.22280226213</v>
       </c>
       <c r="H84">
-        <v>22.01870693488245</v>
+        <v>18.46791472486521</v>
       </c>
       <c r="I84">
-        <v>1428</v>
+        <v>3063</v>
       </c>
     </row>
     <row r="85">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Church Rock Chapter</t>
+          <t>Torreon Chapter</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3157,22 +3157,22 @@
         </is>
       </c>
       <c r="D85">
-        <v>40.47880194142542</v>
+        <v>39.69942347521665</v>
       </c>
       <c r="E85">
-        <v>1.636373562236403</v>
+        <v>1.401860275628119</v>
       </c>
       <c r="F85">
-        <v>5.817439045625099E-05</v>
+        <v>4.983725533187032E-05</v>
       </c>
       <c r="G85">
-        <v>56567.22280226213</v>
+        <v>32113.33366607936</v>
       </c>
       <c r="H85">
-        <v>18.46791472486521</v>
+        <v>19.35704259558732</v>
       </c>
       <c r="I85">
-        <v>3063</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="86">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Torreon Chapter</t>
+          <t>Casamero Lake Chapter</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3190,22 +3190,22 @@
         </is>
       </c>
       <c r="D86">
-        <v>40.47630639187165</v>
+        <v>39.43378265429456</v>
       </c>
       <c r="E86">
-        <v>1.401860275628119</v>
+        <v>0.9673459632626169</v>
       </c>
       <c r="F86">
-        <v>4.983725533187032E-05</v>
+        <v>3.438992359190159E-05</v>
       </c>
       <c r="G86">
-        <v>32113.33366607936</v>
+        <v>7171.626628607789</v>
       </c>
       <c r="H86">
-        <v>19.35704259558732</v>
+        <v>16.83480429250655</v>
       </c>
       <c r="I86">
-        <v>1659</v>
+        <v>426</v>
       </c>
     </row>
     <row r="87">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Casamero Lake Chapter</t>
+          <t>Fruitland Chapter</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3223,22 +3223,22 @@
         </is>
       </c>
       <c r="D87">
-        <v>40.37264661785358</v>
+        <v>38.92530693542288</v>
       </c>
       <c r="E87">
-        <v>0.9673459632626169</v>
+        <v>1.864425111665208</v>
       </c>
       <c r="F87">
-        <v>3.438992359190159E-05</v>
+        <v>6.628180564969429E-05</v>
       </c>
       <c r="G87">
-        <v>7171.626628607789</v>
+        <v>55809.64630231838</v>
       </c>
       <c r="H87">
-        <v>16.83480429250655</v>
+        <v>21.56477832392518</v>
       </c>
       <c r="I87">
-        <v>426</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="88">
@@ -3247,7 +3247,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Fruitland Chapter</t>
+          <t>Nenahnezad/San Juan Chapter</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3256,22 +3256,22 @@
         </is>
       </c>
       <c r="D88">
-        <v>39.54829687583464</v>
+        <v>38.4998468669022</v>
       </c>
       <c r="E88">
-        <v>1.864425111665208</v>
+        <v>1.530492856645816</v>
       </c>
       <c r="F88">
-        <v>6.628180564969429E-05</v>
+        <v>5.441024658900839E-05</v>
       </c>
       <c r="G88">
-        <v>55809.64630231838</v>
+        <v>31480.09215920649</v>
       </c>
       <c r="H88">
-        <v>21.56477832392518</v>
+        <v>20.46820036359329</v>
       </c>
       <c r="I88">
-        <v>2588</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="89">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Nenahnezad/San Juan Chapter</t>
+          <t>Cameron Chapter</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3289,22 +3289,22 @@
         </is>
       </c>
       <c r="D89">
-        <v>39.28084229767148</v>
+        <v>38.33301835496885</v>
       </c>
       <c r="E89">
-        <v>1.530492856645816</v>
+        <v>1.527488502903494</v>
       </c>
       <c r="F89">
-        <v>5.441024658900839E-05</v>
+        <v>5.430343940774608E-05</v>
       </c>
       <c r="G89">
-        <v>31480.09215920649</v>
+        <v>20886.79451749201</v>
       </c>
       <c r="H89">
-        <v>20.46820036359329</v>
+        <v>22.43479540009883</v>
       </c>
       <c r="I89">
-        <v>1538</v>
+        <v>931</v>
       </c>
     </row>
     <row r="90">
@@ -3322,7 +3322,7 @@
         </is>
       </c>
       <c r="D90">
-        <v>39.27461260634612</v>
+        <v>38.32298105444637</v>
       </c>
       <c r="E90">
         <v>1.174265310704007</v>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Cameron Chapter</t>
+          <t>Twin Lakes Chapter</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3355,22 +3355,22 @@
         </is>
       </c>
       <c r="D91">
-        <v>39.18281073855267</v>
+        <v>38.03645399321642</v>
       </c>
       <c r="E91">
-        <v>1.527488502903494</v>
+        <v>1.756529396110181</v>
       </c>
       <c r="F91">
-        <v>5.430343940774608E-05</v>
+        <v>6.244602656470567E-05</v>
       </c>
       <c r="G91">
-        <v>20886.79451749201</v>
+        <v>44446.23517518774</v>
       </c>
       <c r="H91">
-        <v>22.43479540009883</v>
+        <v>21.17495720590173</v>
       </c>
       <c r="I91">
-        <v>931</v>
+        <v>2099</v>
       </c>
     </row>
     <row r="92">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Twin Lakes Chapter</t>
+          <t>Nazlini Chapter</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3388,22 +3388,22 @@
         </is>
       </c>
       <c r="D92">
-        <v>38.73324229987504</v>
+        <v>37.51736758069296</v>
       </c>
       <c r="E92">
-        <v>1.756529396110181</v>
+        <v>1.438832693007208</v>
       </c>
       <c r="F92">
-        <v>6.244602656470567E-05</v>
+        <v>5.115165437519337E-05</v>
       </c>
       <c r="G92">
-        <v>44446.23517518774</v>
+        <v>23636.2698288828</v>
       </c>
       <c r="H92">
-        <v>21.17495720590173</v>
+        <v>19.53410729659736</v>
       </c>
       <c r="I92">
-        <v>2099</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="93">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Nazlini Chapter</t>
+          <t>Hogback Chapter</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3421,22 +3421,22 @@
         </is>
       </c>
       <c r="D93">
-        <v>38.34930381318389</v>
+        <v>35.94697460591142</v>
       </c>
       <c r="E93">
-        <v>1.438832693007208</v>
+        <v>1.796180553596647</v>
       </c>
       <c r="F93">
-        <v>5.115165437519337E-05</v>
+        <v>6.385565696383499E-05</v>
       </c>
       <c r="G93">
-        <v>23636.2698288828</v>
+        <v>31614.36502313642</v>
       </c>
       <c r="H93">
-        <v>19.53410729659736</v>
+        <v>22.38977692856687</v>
       </c>
       <c r="I93">
-        <v>1210</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="94">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Hogback Chapter</t>
+          <t>Many Farms Chapter</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -3454,22 +3454,22 @@
         </is>
       </c>
       <c r="D94">
-        <v>36.7270980170135</v>
+        <v>35.65812747642896</v>
       </c>
       <c r="E94">
-        <v>1.796180553596647</v>
+        <v>1.916971931174239</v>
       </c>
       <c r="F94">
-        <v>6.385565696383499E-05</v>
+        <v>6.814988715986898E-05</v>
       </c>
       <c r="G94">
-        <v>31614.36502313642</v>
+        <v>50649.64162337014</v>
       </c>
       <c r="H94">
-        <v>22.38977692856687</v>
+        <v>20.22749266109031</v>
       </c>
       <c r="I94">
-        <v>1412</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="95">
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="D95">
-        <v>36.57884745421026</v>
+        <v>35.6496027693794</v>
       </c>
       <c r="E95">
         <v>1.43643539074584</v>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Many Farms Chapter</t>
+          <t>Crownpoint Chapter</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3520,22 +3520,22 @@
         </is>
       </c>
       <c r="D96">
-        <v>36.31462847358875</v>
+        <v>35.36886749513454</v>
       </c>
       <c r="E96">
-        <v>1.916971931174239</v>
+        <v>1.756885326365939</v>
       </c>
       <c r="F96">
-        <v>6.814988715986898E-05</v>
+        <v>6.24586801703074E-05</v>
       </c>
       <c r="G96">
-        <v>50649.64162337014</v>
+        <v>50721.78911346889</v>
       </c>
       <c r="H96">
-        <v>20.22749266109031</v>
+        <v>17.19382681812505</v>
       </c>
       <c r="I96">
-        <v>2504</v>
+        <v>2950</v>
       </c>
     </row>
     <row r="97">
@@ -3544,7 +3544,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Gadii'ahi Chapter</t>
+          <t>Tuba City Chapter</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3553,22 +3553,22 @@
         </is>
       </c>
       <c r="D97">
-        <v>36.10128401461144</v>
+        <v>35.31981988218078</v>
       </c>
       <c r="E97">
-        <v>1.668682136174088</v>
+        <v>2.96235427050619</v>
       </c>
       <c r="F97">
-        <v>5.932298613068052E-05</v>
+        <v>0.0001053140664083115</v>
       </c>
       <c r="G97">
-        <v>11259.17360860693</v>
+        <v>150042.5080682224</v>
       </c>
       <c r="H97">
-        <v>23.65372606850196</v>
+        <v>17.18109562214845</v>
       </c>
       <c r="I97">
-        <v>476</v>
+        <v>8733</v>
       </c>
     </row>
     <row r="98">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Crownpoint Chapter</t>
+          <t>Gadii'ahi Chapter</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3586,22 +3586,22 @@
         </is>
       </c>
       <c r="D98">
-        <v>36.02489993872019</v>
+        <v>35.18896615465692</v>
       </c>
       <c r="E98">
-        <v>1.756885326365939</v>
+        <v>1.668682136174088</v>
       </c>
       <c r="F98">
-        <v>6.24586801703074E-05</v>
+        <v>5.932298613068052E-05</v>
       </c>
       <c r="G98">
-        <v>50721.78911346889</v>
+        <v>11259.17360860693</v>
       </c>
       <c r="H98">
-        <v>17.19382681812505</v>
+        <v>23.65372606850196</v>
       </c>
       <c r="I98">
-        <v>2950</v>
+        <v>476</v>
       </c>
     </row>
     <row r="99">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>San Juan Southern Paiute Southern Area</t>
+          <t>Tonalea Chapter</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3619,22 +3619,22 @@
         </is>
       </c>
       <c r="D99">
-        <v>35.62039489037362</v>
+        <v>34.87725595968259</v>
       </c>
       <c r="E99">
-        <v>1.164236117510514</v>
+        <v>1.888612051611593</v>
       </c>
       <c r="F99">
-        <v>4.138952623431703E-05</v>
+        <v>6.714167073237127E-05</v>
       </c>
       <c r="G99">
-        <v>218.1663433710178</v>
+        <v>47842.74994135223</v>
       </c>
       <c r="H99">
-        <v>16.78202641315522</v>
+        <v>19.53562676249581</v>
       </c>
       <c r="I99">
-        <v>13</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="100">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Tonalea Chapter</t>
+          <t>Chinle Chapter</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3652,22 +3652,22 @@
         </is>
       </c>
       <c r="D100">
-        <v>35.55198599194878</v>
+        <v>33.92565594654577</v>
       </c>
       <c r="E100">
-        <v>1.888612051611593</v>
+        <v>2.86566287883382</v>
       </c>
       <c r="F100">
-        <v>6.714167073237127E-05</v>
+        <v>0.0001018766100091631</v>
       </c>
       <c r="G100">
-        <v>47842.74994135223</v>
+        <v>133949.6650198771</v>
       </c>
       <c r="H100">
-        <v>19.53562676249581</v>
+        <v>17.44817832745566</v>
       </c>
       <c r="I100">
-        <v>2449</v>
+        <v>7677</v>
       </c>
     </row>
     <row r="101">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Tuba City Chapter</t>
+          <t>Ojo Encino Chapter</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3685,22 +3685,22 @@
         </is>
       </c>
       <c r="D101">
-        <v>35.33082534299491</v>
+        <v>33.36859906283025</v>
       </c>
       <c r="E101">
-        <v>2.96235427050619</v>
+        <v>1.45901274382132</v>
       </c>
       <c r="F101">
-        <v>0.0001053140664083115</v>
+        <v>5.186907134071968E-05</v>
       </c>
       <c r="G101">
-        <v>150042.5080682224</v>
+        <v>7212.364062406295</v>
       </c>
       <c r="H101">
-        <v>17.18109562214845</v>
+        <v>19.08032820742406</v>
       </c>
       <c r="I101">
-        <v>8733</v>
+        <v>378</v>
       </c>
     </row>
     <row r="102">
@@ -3709,7 +3709,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Ojo Encino Chapter</t>
+          <t>Thoreau Chapter</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -3718,22 +3718,22 @@
         </is>
       </c>
       <c r="D102">
-        <v>34.30719846181215</v>
+        <v>32.20206427783764</v>
       </c>
       <c r="E102">
-        <v>1.45901274382132</v>
+        <v>1.609699322897919</v>
       </c>
       <c r="F102">
-        <v>5.186907134071968E-05</v>
+        <v>5.722609988849111E-05</v>
       </c>
       <c r="G102">
-        <v>7212.364062406295</v>
+        <v>24636.14815329354</v>
       </c>
       <c r="H102">
-        <v>19.08032820742406</v>
+        <v>16.87407407759832</v>
       </c>
       <c r="I102">
-        <v>378</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="103">
@@ -3742,7 +3742,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Chinle Chapter</t>
+          <t>Smith Lake Chapter</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -3751,22 +3751,22 @@
         </is>
       </c>
       <c r="D103">
-        <v>34.04117452511551</v>
+        <v>31.76370966330672</v>
       </c>
       <c r="E103">
-        <v>2.86566287883382</v>
+        <v>1.795603522603339</v>
       </c>
       <c r="F103">
-        <v>0.0001018766100091631</v>
+        <v>6.383514304996792E-05</v>
       </c>
       <c r="G103">
-        <v>133949.6650198771</v>
+        <v>18541.11161000585</v>
       </c>
       <c r="H103">
-        <v>17.44817832745566</v>
+        <v>20.85614354331366</v>
       </c>
       <c r="I103">
-        <v>7677</v>
+        <v>889</v>
       </c>
     </row>
     <row r="104">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Thoreau Chapter</t>
+          <t>Rock Springs Chapter</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3784,22 +3784,22 @@
         </is>
       </c>
       <c r="D104">
-        <v>33.02750691558296</v>
+        <v>31.25388661501031</v>
       </c>
       <c r="E104">
-        <v>1.609699322897919</v>
+        <v>1.838078122761735</v>
       </c>
       <c r="F104">
-        <v>5.722609988849111E-05</v>
+        <v>6.534514909694335E-05</v>
       </c>
       <c r="G104">
-        <v>24636.14815329354</v>
+        <v>23167.22863367134</v>
       </c>
       <c r="H104">
-        <v>16.87407407759832</v>
+        <v>20.11044152228415</v>
       </c>
       <c r="I104">
-        <v>1460</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="105">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Smith Lake Chapter</t>
+          <t>Becenti Chapter</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3817,22 +3817,22 @@
         </is>
       </c>
       <c r="D105">
-        <v>32.62873581467109</v>
+        <v>31.19497062686148</v>
       </c>
       <c r="E105">
-        <v>1.795603522603339</v>
+        <v>1.575996066186617</v>
       </c>
       <c r="F105">
-        <v>6.383514304996792E-05</v>
+        <v>5.602792212467357E-05</v>
       </c>
       <c r="G105">
-        <v>18541.11161000585</v>
+        <v>9030.073371185117</v>
       </c>
       <c r="H105">
-        <v>20.85614354331366</v>
+        <v>18.50424871144491</v>
       </c>
       <c r="I105">
-        <v>889</v>
+        <v>488</v>
       </c>
     </row>
     <row r="106">
@@ -3841,7 +3841,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Becenti Chapter</t>
+          <t>Bread Springs Chapter</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3850,22 +3850,22 @@
         </is>
       </c>
       <c r="D106">
-        <v>32.12176512185822</v>
+        <v>29.71339575843293</v>
       </c>
       <c r="E106">
-        <v>1.575996066186617</v>
+        <v>1.95078109694033</v>
       </c>
       <c r="F106">
-        <v>5.602792212467357E-05</v>
+        <v>6.935183007539046E-05</v>
       </c>
       <c r="G106">
-        <v>9030.073371185117</v>
+        <v>20866.52376350236</v>
       </c>
       <c r="H106">
-        <v>18.50424871144491</v>
+        <v>20.95032506375739</v>
       </c>
       <c r="I106">
-        <v>488</v>
+        <v>996</v>
       </c>
     </row>
     <row r="107">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Rock Springs Chapter</t>
+          <t>Iyanbito Chapter</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3883,22 +3883,22 @@
         </is>
       </c>
       <c r="D107">
-        <v>32.08886898158209</v>
+        <v>29.38933799678719</v>
       </c>
       <c r="E107">
-        <v>1.838078122761735</v>
+        <v>1.780510238539746</v>
       </c>
       <c r="F107">
-        <v>6.534514909694335E-05</v>
+        <v>6.329856471562806E-05</v>
       </c>
       <c r="G107">
-        <v>23167.22863367134</v>
+        <v>22744.14059812597</v>
       </c>
       <c r="H107">
-        <v>20.11044152228415</v>
+        <v>17.33547301686431</v>
       </c>
       <c r="I107">
-        <v>1152</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="108">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Bread Springs Chapter</t>
+          <t>Kayenta Chapter</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3916,22 +3916,22 @@
         </is>
       </c>
       <c r="D108">
-        <v>30.56331978809646</v>
+        <v>29.00760890838296</v>
       </c>
       <c r="E108">
-        <v>1.95078109694033</v>
+        <v>2.690729273536222</v>
       </c>
       <c r="F108">
-        <v>6.935183007539046E-05</v>
+        <v>9.56575802635382E-05</v>
       </c>
       <c r="G108">
-        <v>20866.52376350236</v>
+        <v>97662.69059229434</v>
       </c>
       <c r="H108">
-        <v>20.95032506375739</v>
+        <v>16.99368202406374</v>
       </c>
       <c r="I108">
-        <v>996</v>
+        <v>5747</v>
       </c>
     </row>
     <row r="109">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Iyanbito Chapter</t>
+          <t>Red Rock Chapter</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3949,22 +3949,22 @@
         </is>
       </c>
       <c r="D109">
-        <v>30.22706805993111</v>
+        <v>26.87074100258636</v>
       </c>
       <c r="E109">
-        <v>1.780510238539746</v>
+        <v>2.107297099587753</v>
       </c>
       <c r="F109">
-        <v>6.329856471562806E-05</v>
+        <v>7.49160992989893E-05</v>
       </c>
       <c r="G109">
-        <v>22744.14059812597</v>
+        <v>37238.79050475307</v>
       </c>
       <c r="H109">
-        <v>17.33547301686431</v>
+        <v>17.36883885482886</v>
       </c>
       <c r="I109">
-        <v>1312</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="110">
@@ -3973,7 +3973,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Kayenta Chapter</t>
+          <t>Coalmine Mesa Chapter</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3982,87 +3982,21 @@
         </is>
       </c>
       <c r="D110">
-        <v>29.35878906769089</v>
+        <v>19.09054092423021</v>
       </c>
       <c r="E110">
-        <v>2.690729273536222</v>
+        <v>2.499455463566132</v>
       </c>
       <c r="F110">
-        <v>9.56575802635382E-05</v>
+        <v>8.88576431574613E-05</v>
       </c>
       <c r="G110">
-        <v>97662.69059229434</v>
+        <v>17820.2671721494</v>
       </c>
       <c r="H110">
-        <v>16.99368202406374</v>
+        <v>20.20438454892222</v>
       </c>
       <c r="I110">
-        <v>5747</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111">
-        <v>110</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Red Rock Chapter</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>Tier 4: Lower Priority</t>
-        </is>
-      </c>
-      <c r="D111">
-        <v>27.61433722946736</v>
-      </c>
-      <c r="E111">
-        <v>2.107297099587753</v>
-      </c>
-      <c r="F111">
-        <v>7.49160992989893E-05</v>
-      </c>
-      <c r="G111">
-        <v>37238.79050475307</v>
-      </c>
-      <c r="H111">
-        <v>17.36883885482886</v>
-      </c>
-      <c r="I111">
-        <v>2144</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112">
-        <v>111</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>Coalmine Mesa Chapter</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Tier 4: Lower Priority</t>
-        </is>
-      </c>
-      <c r="D112">
-        <v>19.96024851686576</v>
-      </c>
-      <c r="E112">
-        <v>2.499455463566132</v>
-      </c>
-      <c r="F112">
-        <v>8.88576431574613E-05</v>
-      </c>
-      <c r="G112">
-        <v>17820.2671721494</v>
-      </c>
-      <c r="H112">
-        <v>20.20438454892222</v>
-      </c>
-      <c r="I112">
         <v>882</v>
       </c>
     </row>
@@ -4118,16 +4052,16 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>-0.2768690768690769</v>
+        <v>-0.291715318320823</v>
       </c>
       <c r="D2">
-        <v>0.9587353401958733</v>
+        <v>0.956421816439775</v>
       </c>
       <c r="E2">
-        <v>0.3138695101963854</v>
+        <v>0.3084679008311121</v>
       </c>
       <c r="F2">
-        <v>0.3138695101963854</v>
+        <v>0.3084679008311121</v>
       </c>
     </row>
     <row r="3">
@@ -4137,19 +4071,19 @@
         </is>
       </c>
       <c r="B3">
-        <v>-0.2768690768690769</v>
+        <v>-0.291715318320823</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>-0.4837595812594003</v>
+        <v>-0.5092415403703093</v>
       </c>
       <c r="E3">
-        <v>-0.4770655087739061</v>
+        <v>-0.4633227534084084</v>
       </c>
       <c r="F3">
-        <v>-0.4770655087739061</v>
+        <v>-0.4633227534084084</v>
       </c>
     </row>
     <row r="4">
@@ -4159,19 +4093,19 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.9587353401958733</v>
+        <v>0.956421816439775</v>
       </c>
       <c r="C4">
-        <v>-0.4837595812594003</v>
+        <v>-0.5092415403703093</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4">
-        <v>0.3702179381498258</v>
+        <v>0.3671958260984531</v>
       </c>
       <c r="F4">
-        <v>0.3702179381498258</v>
+        <v>0.3671958260984531</v>
       </c>
     </row>
     <row r="5">
@@ -4181,13 +4115,13 @@
         </is>
       </c>
       <c r="B5">
-        <v>0.3138695101963854</v>
+        <v>0.3084679008311121</v>
       </c>
       <c r="C5">
-        <v>-0.4770655087739061</v>
+        <v>-0.4633227534084084</v>
       </c>
       <c r="D5">
-        <v>0.3702179381498258</v>
+        <v>0.3671958260984531</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -4203,13 +4137,13 @@
         </is>
       </c>
       <c r="B6">
-        <v>0.3138695101963854</v>
+        <v>0.3084679008311121</v>
       </c>
       <c r="C6">
-        <v>-0.4770655087739061</v>
+        <v>-0.4633227534084084</v>
       </c>
       <c r="D6">
-        <v>0.3702179381498258</v>
+        <v>0.3671958260984531</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -4262,16 +4196,16 @@
         </is>
       </c>
       <c r="B2">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2">
-        <v>55859</v>
+        <v>55846</v>
       </c>
       <c r="D2">
-        <v>1041187.097441337</v>
+        <v>1040968.931097966</v>
       </c>
       <c r="E2">
-        <v>1.787885617111537</v>
+        <v>1.81098374672639</v>
       </c>
     </row>
     <row r="3">
@@ -4300,16 +4234,16 @@
         </is>
       </c>
       <c r="B4">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4">
-        <v>48926</v>
+        <v>47959</v>
       </c>
       <c r="D4">
-        <v>1024540.275660842</v>
+        <v>999191.2395509498</v>
       </c>
       <c r="E4">
-        <v>0.7302910643222045</v>
+        <v>0.7387575197493456</v>
       </c>
     </row>
     <row r="5">
@@ -4322,13 +4256,13 @@
         <v>28</v>
       </c>
       <c r="C5">
-        <v>26031</v>
+        <v>26971</v>
       </c>
       <c r="D5">
-        <v>650479.3946040373</v>
+        <v>674998.0959821753</v>
       </c>
       <c r="E5">
-        <v>0.2030939161501801</v>
+        <v>0.2210116578569443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>